<commit_message>
feat(simulator): return ScanDataResult with unit info instead of raw values
Changed read_channel_measurement() and read_all_channels() to return
structured ScanDataResult objects containing value, unit, full_unit,
and range_info instead of plain float values. Added _get_unit_info()
helper method to map measurement types to their corresponding units.
This provides more complete simulation data matching the real instrument's
output format.
</commit_message>
<xml_diff>
--- a/B1ControlExtensionBoardv232_2026-01-30.xlsx
+++ b/B1ControlExtensionBoardv232_2026-01-30.xlsx
@@ -31,18 +31,12 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -77,14 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,14 +447,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="221" customWidth="1" min="2" max="2"/>
+    <col width="262" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="5" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
@@ -555,38 +548,38 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>FAILED CH2 (5.0VD): -0.0002452 (expected: 2.0 - 2.1); CH3 (12V): -0.0002955 (expected: 2.0 - 2.1); CH4 (7V): -0.0003076 (expected: 2.0 - 2.1); CH6: -0.0003198 (expected: 2.1 - 2.2); CH7: -0.0003656 (expected: 1.0 - 1.1)</t>
+          <t>FAILED CH1 (3.3VD): 5.0429797 (expected: 3.2 - 3.4); CH2 (5.0VD): 4.9584135 (expected: 2.0 - 2.1); CH3 (12V): 5.0366938 (expected: 2.0 - 2.1); CH4 (7V): 5.0932652 (expected: 2.0 - 2.1); CH6: 4.9238724 (expected: 2.1 - 2.2); CH7: 4.9855825 (expected: 1.0 - 1.1)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>3.2960139</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>-0.0002452</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>-0.0002955</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>-0.0003076</t>
+          <t>5.0429797</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>4.9584135</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>5.0366938</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>5.0932652</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>-0.0003198</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>-0.0003656</t>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>4.9238724</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>4.9855825</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -596,7 +589,7 @@
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-30 11:23:55</t>
+          <t>2026-01-30 12:19:33</t>
         </is>
       </c>
     </row>

</xml_diff>